<commit_message>
Agregue una CNN para predecir
</commit_message>
<xml_diff>
--- a/Docs/ConfiguracionRealModelo.xlsx
+++ b/Docs/ConfiguracionRealModelo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabia\Desktop\Universidad\TesisML\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17F86C60-0DCE-4BA2-BC80-6B1C4B35E140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F9227D9-B230-4F29-9DD0-3FEB79183B5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EB321E2F-A158-4D4F-98D8-E5A615C233E9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{EB321E2F-A158-4D4F-98D8-E5A615C233E9}"/>
   </bookViews>
   <sheets>
     <sheet name="LSTM Clasica " sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
   <si>
     <t>Descripcion</t>
   </si>
@@ -440,6 +440,12 @@
   </si>
   <si>
     <t>LSTM Clasica con ventanas de tiempo de 90 dias: Close, Volumen, RSI, MACD, ATR, EMA20, EMA51</t>
+  </si>
+  <si>
+    <t>LSTM Clasica con ventanas de tiempo de 90 dias: Close, Volumen, RSI, MACD, ATR, EMA20, EMA52</t>
+  </si>
+  <si>
+    <t>LSTM Bidireccional con ventanas de tiempo de 90 dias: Close, Volumen, RSI, MACD, ATR, EMA20, EMA52</t>
   </si>
 </sst>
 </file>
@@ -494,7 +500,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -508,7 +514,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -551,9 +556,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{17DD9F00-2A82-4A5D-A129-DC1A3966A506}" name="Tabla1" displayName="Tabla1" ref="B1:E14" totalsRowShown="0">
   <autoFilter ref="B1:E14" xr:uid="{17DD9F00-2A82-4A5D-A129-DC1A3966A506}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{A219EF1F-5F03-44BB-94D9-DDF84B5D15C2}" name="Descripcion" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{F2DDE521-31A0-4967-A63D-8E3F5E6ED67C}" name=" Caracteristicas" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{2FB7966A-C401-40F8-9DC1-33ADC97693CD}" name="Fecha de ejecucion" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{A219EF1F-5F03-44BB-94D9-DDF84B5D15C2}" name="Descripcion" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{F2DDE521-31A0-4967-A63D-8E3F5E6ED67C}" name=" Caracteristicas" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{2FB7966A-C401-40F8-9DC1-33ADC97693CD}" name="Fecha de ejecucion" dataDxfId="3"/>
     <tableColumn id="4" xr3:uid="{A19B35B0-35FB-4491-9788-07CC4387A7B2}" name="Grafica"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -564,9 +569,9 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{76FB69AF-82F3-47A8-80EA-3563E28A1970}" name="Tabla13" displayName="Tabla13" ref="B1:E14" totalsRowShown="0">
   <autoFilter ref="B1:E14" xr:uid="{76FB69AF-82F3-47A8-80EA-3563E28A1970}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{0A114052-5782-45CC-9E5D-CC04A9FD2372}" name="Descripcion" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{9F71BC4A-3F7C-4E8A-AF6E-2CD68C6A137B}" name=" Caracteristicas" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{E6F6E4ED-91D0-4818-8F23-52323C2D1126}" name="Fecha de ejecucion" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{0A114052-5782-45CC-9E5D-CC04A9FD2372}" name="Descripcion" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{9F71BC4A-3F7C-4E8A-AF6E-2CD68C6A137B}" name=" Caracteristicas" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{E6F6E4ED-91D0-4818-8F23-52323C2D1126}" name="Fecha de ejecucion" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{0B1A018E-7C86-49CD-A15E-3842F058E12A}" name="Grafica"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -890,7 +895,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A369B6B-CB39-4503-91B5-AD035AF9D5C3}">
-  <dimension ref="B1:I14"/>
+  <dimension ref="B1:E14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="21" customWidth="1"/>
@@ -898,7 +903,7 @@
     <col min="4" max="4" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9">
+    <row r="1" spans="2:5">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -912,7 +917,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="2:9" ht="129.6">
+    <row r="2" spans="2:5" ht="129.6">
       <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
@@ -926,7 +931,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="129.6">
+    <row r="3" spans="2:5" ht="129.6">
       <c r="B3" s="1" t="s">
         <v>17</v>
       </c>
@@ -939,59 +944,67 @@
       <c r="E3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="5"/>
-    </row>
-    <row r="4" spans="2:9">
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="2"/>
-    </row>
-    <row r="5" spans="2:9">
+    </row>
+    <row r="4" spans="2:5" ht="129.6">
+      <c r="B4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2">
+        <v>46116.984027777777</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="2"/>
     </row>
-    <row r="6" spans="2:9">
+    <row r="6" spans="2:5">
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="2"/>
     </row>
-    <row r="7" spans="2:9">
+    <row r="7" spans="2:5">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="2"/>
     </row>
-    <row r="8" spans="2:9">
+    <row r="8" spans="2:5">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="2"/>
     </row>
-    <row r="9" spans="2:9">
+    <row r="9" spans="2:5">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="2:9">
+    <row r="10" spans="2:5">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="2"/>
     </row>
-    <row r="11" spans="2:9">
+    <row r="11" spans="2:5">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="2:9">
+    <row r="12" spans="2:5">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="2"/>
     </row>
-    <row r="13" spans="2:9">
+    <row r="13" spans="2:5">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="2:9">
+    <row r="14" spans="2:5">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="2"/>
@@ -1057,15 +1070,25 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="2:5">
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="2"/>
+    <row r="4" spans="2:5" ht="244.8">
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2">
+        <v>46116</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="2"/>
+      <c r="E5" s="4"/>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" s="1"/>

</xml_diff>